<commit_message>
Resume opens in new tab, clearer WATCH cards, model rewritten in plain voice with chart
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NEO_Ramp_Model_Tristan_Massicotte.xlsx
+++ b/NEO_Ramp_Model_Tristan_Massicotte.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tristanmassicotte/Desktop/internship-2027/companies/1x/site/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tristanmassicotte/Desktop/internship-2027/companies/1x/model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0B54B8-A4DB-C640-A9D4-6D41DFE6B0B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{817D9FEB-0D10-954B-9624-ECAC0B45AE09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -33,47 +33,44 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="107">
-  <si>
-    <t>NEO Factory Ramp Model — 10k to 100k robots/yr</t>
-  </si>
-  <si>
-    <t>Prepared by Tristan Massicotte (U of T Industrial Engineering) · October 2026 · ILLUSTRATIVE — built only from public information</t>
-  </si>
-  <si>
-    <t>What this is</t>
-  </si>
-  <si>
-    <t>A small planning model showing what the NEO ramp means on the floor: takt time, motor-line pace, station count, clear-to-build and the excess/obsolete (E&amp;O) risk of a mid-ramp BOM change.</t>
-  </si>
-  <si>
-    <t>What this is NOT</t>
-  </si>
-  <si>
-    <t>It contains no 1X internal data. Every yellow cell is an assumption or placeholder. Replace them with real numbers and every result recalculates.</t>
-  </si>
-  <si>
-    <t>Legend</t>
-  </si>
-  <si>
-    <t>Blue text = input you can change · Yellow fill = key assumption to replace with real data · Black = formula · Green = formula pulling from another tab</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="97">
+  <si>
+    <t>NEO Factory ramp model: 10k to 100k robots a year</t>
+  </si>
+  <si>
+    <t>Tristan Massicotte, U of T Industrial Engineering, October 2026. Built from public information only, so every 1X-specific number in here is my estimate.</t>
+  </si>
+  <si>
+    <t>What it does</t>
+  </si>
+  <si>
+    <t>I built this to see what the ramp means on the floor: takt, motor-line pace, how many stations you'd need, clear-to-build, and how much old stock a mid-ramp part change could leave behind.</t>
+  </si>
+  <si>
+    <t>What's real</t>
+  </si>
+  <si>
+    <t>There is no 1X internal data in here. Yellow cells are my assumptions. Put your real numbers in and everything recalculates.</t>
+  </si>
+  <si>
+    <t>Colours</t>
+  </si>
+  <si>
+    <t>Blue = input, change it. Yellow = my assumption, replace it. Black = formula. Green = formula pulling from another tab.</t>
   </si>
   <si>
     <t>Tabs</t>
   </si>
   <si>
-    <t>Inputs → Takt → Station Sizing → Clear-to-Build → BOM Change</t>
-  </si>
-  <si>
-    <t>Public sources</t>
+    <t>Inputs, Takt, Station Sizing, Clear-to-Build, BOM Change</t>
+  </si>
+  <si>
+    <t>Where the public numbers come from</t>
   </si>
   <si>
     <t>Capacity 10k/yr, target 100k+/yr by end 2027</t>
@@ -94,22 +91,16 @@
     <t>humanoid.guide NEO spec sheet (launch spec, Oct 2025). New 25-DoF hands announced Jul 9 2026 may change the count.</t>
   </si>
   <si>
-    <t>10,000 hands targeted in 2026</t>
-  </si>
-  <si>
-    <t>1X 'NEO's Hands' announcement (Jul 9 2026), as reported by humanoid.guide and Noqta</t>
-  </si>
-  <si>
     <t>Five commodity areas</t>
   </si>
   <si>
     <t>1X job posting 'Supply Chain Planner – Advanced Robotics Commodities' (1x.tech/open-positions)</t>
   </si>
   <si>
-    <t>Inputs &amp; assumptions</t>
-  </si>
-  <si>
-    <t>Change blue cells. Yellow = assumption that should be replaced with real 1X data.</t>
+    <t>Inputs</t>
+  </si>
+  <si>
+    <t>Change the blue cells. The yellow ones are my guesses; replace them with real numbers if you have them.</t>
   </si>
   <si>
     <t>Parameter</t>
@@ -121,7 +112,7 @@
     <t>Unit</t>
   </si>
   <si>
-    <t>Basis / source</t>
+    <t>Where it comes from</t>
   </si>
   <si>
     <t>Working days per year</t>
@@ -130,7 +121,7 @@
     <t>days</t>
   </si>
   <si>
-    <t>Assumption: 5-day weeks, 50 weeks</t>
+    <t>My assumption: 5-day weeks, 50 weeks a year</t>
   </si>
   <si>
     <t>Shifts per day</t>
@@ -139,7 +130,7 @@
     <t>shifts</t>
   </si>
   <si>
-    <t>Assumption</t>
+    <t>My assumption</t>
   </si>
   <si>
     <t>Hours per shift</t>
@@ -154,7 +145,7 @@
     <t>%</t>
   </si>
   <si>
-    <t>Assumption: 100% gives the theoretical takt. Set ~0.85–0.90 for breaks, changeovers, downtime</t>
+    <t>100% gives the theoretical takt. I'd use 85 to 90% once breaks, changeovers and downtime are in.</t>
   </si>
   <si>
     <t>Actuated joints (≈ motors) per robot</t>
@@ -163,22 +154,7 @@
     <t>motors</t>
   </si>
   <si>
-    <t>Public spec: 75 DoF (humanoid.guide). Assumes 1 motor per actuated joint</t>
-  </si>
-  <si>
-    <t>Hands per robot</t>
-  </si>
-  <si>
-    <t>hands</t>
-  </si>
-  <si>
-    <t>Physical</t>
-  </si>
-  <si>
-    <t>Hands targeted for 2026 (public)</t>
-  </si>
-  <si>
-    <t>1X hand announcement, Jul 9 2026</t>
+    <t>75 DoF from the public spec (humanoid.guide). I'm assuming one motor per joint.</t>
   </si>
   <si>
     <t>Final-assembly work content per robot</t>
@@ -187,13 +163,13 @@
     <t>labour-min</t>
   </si>
   <si>
-    <t>PLACEHOLDER — no public data. Replace with real routing time</t>
+    <t>No public number, so this is a placeholder. The real routing time goes here.</t>
   </si>
   <si>
     <t>Line balance efficiency</t>
   </si>
   <si>
-    <t>Assumption: typical manual line</t>
+    <t>My assumption for a manual line</t>
   </si>
   <si>
     <t>Automated motor-cell cycle time</t>
@@ -202,7 +178,7 @@
     <t>sec / motor</t>
   </si>
   <si>
-    <t>PLACEHOLDER — no public data</t>
+    <t>No public number, so this is a placeholder.</t>
   </si>
   <si>
     <t>Available hours per year</t>
@@ -211,10 +187,10 @@
     <t>Days × shifts × hours × availability</t>
   </si>
   <si>
-    <t>Takt time at each ramp step</t>
-  </si>
-  <si>
-    <t>Takt = available time ÷ demand. The pace one station must hit for the line to meet volume.</t>
+    <t>Takt at each ramp step</t>
+  </si>
+  <si>
+    <t>Takt = available time ÷ demand: how often a finished robot has to come off the line.</t>
   </si>
   <si>
     <t>Annual volume (robots/yr)</t>
@@ -232,28 +208,19 @@
     <t>Motor takt (sec)</t>
   </si>
   <si>
-    <t>Hands per year needed</t>
-  </si>
-  <si>
-    <t>Hands needed ÷ 2026 hand target</t>
-  </si>
-  <si>
-    <t>Shift-pattern sensitivity at 100,000 robots/yr (robot takt, min)</t>
+    <t>What the shift pattern does at 100,000 robots a year</t>
   </si>
   <si>
     <t>Available h/yr</t>
   </si>
   <si>
-    <t>Reading: going from 10k to 100k/yr cuts robot takt 10×. The motor line feels it most: ~75 motors per robot means a motor every ~2 s at 100k on two shifts.</t>
-  </si>
-  <si>
-    <t>Hands check: if the 10,000-hand 2026 target counts single hands, it covers ~5,000 robots (2 hands each). Worth confirming how it is counted.</t>
-  </si>
-  <si>
-    <t>What the takt means for the floor</t>
-  </si>
-  <si>
-    <t>Manual stations = work content ÷ (takt × balance efficiency). Motor cells = cell cycle ÷ motor takt. Both rounded up.</t>
+    <t>Going from 10k to 100k a year makes the takt 10 times shorter. The motor lines feel it most, since each robot needs about 75 motors.</t>
+  </si>
+  <si>
+    <t>Stations needed at each step</t>
+  </si>
+  <si>
+    <t>Manual stations = work content ÷ (takt × balance efficiency), rounded up. Same idea for the motor cells.</t>
   </si>
   <si>
     <t>Manual assembly stations needed</t>
@@ -262,13 +229,13 @@
     <t>Automated motor cells needed</t>
   </si>
   <si>
-    <t>Work content and motor-cell cycle are placeholders (yellow on Inputs). The point is the scaling: ~10× the stations or cells for the same design, which is why the ramp is an automation and line-design problem, not just more people.</t>
+    <t>Work content and cell cycle time are placeholders, so look at the scaling more than the exact counts: same design, about 10 times the stations.</t>
   </si>
   <si>
     <t>Clear-to-build: how many robots can we start today?</t>
   </si>
   <si>
-    <t>Buildable = MIN over commodities of FLOOR(on-hand kits ÷ kits per robot). Example quantities only.</t>
+    <t>The scarcest commodity sets the answer. The quantities are made up for the example.</t>
   </si>
   <si>
     <t>Commodity area (from 1X job posting)</t>
@@ -283,7 +250,7 @@
     <t>Robots buildable</t>
   </si>
   <si>
-    <t>Is constraint?</t>
+    <t>Constraint</t>
   </si>
   <si>
     <t>Motors, PCBs &amp; batteries</t>
@@ -310,13 +277,13 @@
     <t>Weeks of coverage</t>
   </si>
   <si>
-    <t>Example values only. A 'hand mechanisms' line at 2 kits per robot is often where the constraint hides: the per-robot quantity doubles the pull on supply.</t>
-  </si>
-  <si>
-    <t>Mid-ramp BOM change: excess &amp; obsolete (E&amp;O) exposure</t>
-  </si>
-  <si>
-    <t>Example: an old-revision hand module is replaced at a cut-in week. Stock left at cut-in becomes E&amp;O. Change the cut-in week and receipts to see the trade-off.</t>
+    <t>Made-up quantities. I'd look at hand mechanisms first: at 2 kits per robot, they run out twice as fast.</t>
+  </si>
+  <si>
+    <t>New hand revision: how much old stock is left?</t>
+  </si>
+  <si>
+    <t>Old-revision parts still on hand after the cut-in week become excess. Try moving the cut-in week or the open POs.</t>
   </si>
   <si>
     <t>Old-revision parts on hand at week 1</t>
@@ -361,17 +328,16 @@
     <t>E&amp;O exposure ($)</t>
   </si>
   <si>
-    <t>Reading: receipts already on order after the cut-in decision are what turn a design improvement into a write-off. Pulling cut-in earlier, or cancelling/pushing POs inside the supplier's window, is the planning lever.</t>
+    <t>The write-off comes from old-part POs still landing after the cut-in decision. The levers I'd look at: cut in earlier, or cancel or push POs while they're still inside the supplier's window.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="165" formatCode="0.0\x"/>
-    <numFmt numFmtId="166" formatCode="\$#,##0"/>
+    <numFmt numFmtId="165" formatCode="\$#,##0"/>
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
     <font>
@@ -379,7 +345,7 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -459,13 +425,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F2937"/>
-        <bgColor rgb="FF333300"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -496,7 +460,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -513,95 +477,26 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFBFBFBF"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF555555"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF1F2937"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -613,15 +508,243 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="1"/>
+  <c:style val="2"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Manual assembly stations needed</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="1"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Station Sizing'!$C$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Manual assembly stations needed</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="1"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Station Sizing'!$A$5:$A$8</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>10000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>25000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>50000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>100000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Station Sizing'!$C$5:$C$8</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>111</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>221</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>442</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-CE6D-5247-B442-ADA01AF00D37}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="10"/>
+        <c:axId val="100"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="10"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Robots per year</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="1"/>
+        </c:title>
+        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="100"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="1"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="100"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Stations</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="1"/>
+        </c:title>
+        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="10"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5760000" cy="2700000"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:srgbClr val="000000"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -659,128 +782,234 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme>
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="35000">
               <a:schemeClr val="phClr">
                 <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect/>
         </a:gradFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
                 <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
         <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="40000">
               <a:schemeClr val="phClr">
                 <a:tint val="45000"/>
                 <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect/>
         </a:gradFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="80000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="30000"/>
+                <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -792,8 +1021,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
     <col min="2" max="2" width="100" customWidth="1"/>
@@ -825,7 +1054,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
@@ -883,24 +1112,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -910,442 +1130,367 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>24</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B5" s="7">
         <v>250</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B6" s="7">
         <v>2</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B7" s="7">
         <v>8</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="27" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B8" s="9">
         <v>1</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B9" s="7">
         <v>75</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="10">
+        <v>900</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>41</v>
-      </c>
-      <c r="B10" s="10">
-        <v>2</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11" s="11">
-        <v>10000</v>
+        <v>42</v>
+      </c>
+      <c r="B11" s="9">
+        <v>0.85</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="7">
+        <v>30</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="12">
-        <v>900</v>
-      </c>
-      <c r="C12" s="6" t="s">
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D12" s="8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" s="9">
-        <v>0.85</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B14" s="7">
-        <v>30</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B15" s="13">
+      <c r="B13" s="11">
         <f>B5*B6*B7*B8</f>
         <v>4000</v>
       </c>
-      <c r="C15" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="14" t="s">
-        <v>55</v>
+      <c r="C13" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="11">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="13">
         <v>10000</v>
       </c>
-      <c r="B5" s="15">
-        <f>Inputs!$B$15*60/A5</f>
+      <c r="B5" s="14">
+        <f>Inputs!$B$13*60/A5</f>
         <v>24</v>
       </c>
-      <c r="C5" s="15">
-        <f>A5/Inputs!$B$15</f>
+      <c r="C5" s="14">
+        <f>A5/Inputs!$B$13</f>
         <v>2.5</v>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="15">
         <f>A5*Inputs!$B$9</f>
         <v>750000</v>
       </c>
-      <c r="E5" s="17">
-        <f>Inputs!$B$15*3600/D5</f>
+      <c r="E5" s="16">
+        <f>Inputs!$B$13*3600/D5</f>
         <v>19.2</v>
       </c>
-      <c r="F5" s="16">
-        <f>A5*Inputs!$B$10</f>
-        <v>20000</v>
-      </c>
-      <c r="G5" s="18">
-        <f>F5/Inputs!$B$11</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="11">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="13">
         <v>25000</v>
       </c>
-      <c r="B6" s="15">
-        <f>Inputs!$B$15*60/A6</f>
+      <c r="B6" s="14">
+        <f>Inputs!$B$13*60/A6</f>
         <v>9.6</v>
       </c>
-      <c r="C6" s="15">
-        <f>A6/Inputs!$B$15</f>
+      <c r="C6" s="14">
+        <f>A6/Inputs!$B$13</f>
         <v>6.25</v>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="15">
         <f>A6*Inputs!$B$9</f>
         <v>1875000</v>
       </c>
-      <c r="E6" s="17">
-        <f>Inputs!$B$15*3600/D6</f>
+      <c r="E6" s="16">
+        <f>Inputs!$B$13*3600/D6</f>
         <v>7.68</v>
       </c>
-      <c r="F6" s="16">
-        <f>A6*Inputs!$B$10</f>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="13">
         <v>50000</v>
       </c>
-      <c r="G6" s="18">
-        <f>F6/Inputs!$B$11</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="11">
-        <v>50000</v>
-      </c>
-      <c r="B7" s="15">
-        <f>Inputs!$B$15*60/A7</f>
+      <c r="B7" s="14">
+        <f>Inputs!$B$13*60/A7</f>
         <v>4.8</v>
       </c>
-      <c r="C7" s="15">
-        <f>A7/Inputs!$B$15</f>
+      <c r="C7" s="14">
+        <f>A7/Inputs!$B$13</f>
         <v>12.5</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="15">
         <f>A7*Inputs!$B$9</f>
         <v>3750000</v>
       </c>
-      <c r="E7" s="17">
-        <f>Inputs!$B$15*3600/D7</f>
+      <c r="E7" s="16">
+        <f>Inputs!$B$13*3600/D7</f>
         <v>3.84</v>
       </c>
-      <c r="F7" s="16">
-        <f>A7*Inputs!$B$10</f>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="13">
         <v>100000</v>
       </c>
-      <c r="G7" s="18">
-        <f>F7/Inputs!$B$11</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="11">
-        <v>100000</v>
-      </c>
-      <c r="B8" s="15">
-        <f>Inputs!$B$15*60/A8</f>
+      <c r="B8" s="14">
+        <f>Inputs!$B$13*60/A8</f>
         <v>2.4</v>
       </c>
-      <c r="C8" s="15">
-        <f>A8/Inputs!$B$15</f>
+      <c r="C8" s="14">
+        <f>A8/Inputs!$B$13</f>
         <v>25</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="15">
         <f>A8*Inputs!$B$9</f>
         <v>7500000</v>
       </c>
-      <c r="E8" s="17">
-        <f>Inputs!$B$15*3600/D8</f>
+      <c r="E8" s="16">
+        <f>Inputs!$B$13*3600/D8</f>
         <v>1.92</v>
       </c>
-      <c r="F8" s="16">
-        <f>A8*Inputs!$B$10</f>
-        <v>200000</v>
-      </c>
-      <c r="G8" s="18">
-        <f>F8/Inputs!$B$11</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="10">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="17">
         <v>1</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="15">
         <f>Inputs!$B$5*A12*Inputs!$B$7*Inputs!$B$8</f>
         <v>2000</v>
       </c>
-      <c r="C12" s="19">
+      <c r="C12" s="18">
         <f>B12*60/100000</f>
         <v>1.2</v>
       </c>
-      <c r="D12" s="17">
+      <c r="D12" s="16">
         <f>B12*3600/(100000*Inputs!$B$9)</f>
         <v>0.96</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="10">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="17">
         <v>2</v>
       </c>
-      <c r="B13" s="16">
+      <c r="B13" s="15">
         <f>Inputs!$B$5*A13*Inputs!$B$7*Inputs!$B$8</f>
         <v>4000</v>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="18">
         <f>B13*60/100000</f>
         <v>2.4</v>
       </c>
-      <c r="D13" s="17">
+      <c r="D13" s="16">
         <f>B13*3600/(100000*Inputs!$B$9)</f>
         <v>1.92</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="10">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="17">
         <v>3</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="15">
         <f>Inputs!$B$5*A14*Inputs!$B$7*Inputs!$B$8</f>
         <v>6000</v>
       </c>
-      <c r="C14" s="19">
+      <c r="C14" s="18">
         <f>B14*60/100000</f>
         <v>3.6</v>
       </c>
-      <c r="D14" s="17">
+      <c r="D14" s="16">
         <f>B14*3600/(100000*Inputs!$B$9)</f>
         <v>2.88</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="20" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="20" t="s">
-        <v>68</v>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="19" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -1356,134 +1501,134 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="D4" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>72</v>
-      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="16">
+      <c r="A5" s="15">
         <f>Takt!A5</f>
         <v>10000</v>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="14">
         <f>Takt!B5</f>
         <v>24</v>
       </c>
-      <c r="C5" s="16">
-        <f>ROUNDUP(Inputs!$B$12/(B5*Inputs!$B$13),0)</f>
+      <c r="C5" s="15">
+        <f>ROUNDUP(Inputs!$B$10/(B5*Inputs!$B$11),0)</f>
         <v>45</v>
       </c>
-      <c r="D5" s="17">
+      <c r="D5" s="16">
         <f>Takt!E5</f>
         <v>19.2</v>
       </c>
-      <c r="E5" s="16">
-        <f>ROUNDUP(Inputs!$B$14/D5,0)</f>
+      <c r="E5" s="15">
+        <f>ROUNDUP(Inputs!$B$12/D5,0)</f>
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="16">
+      <c r="A6" s="15">
         <f>Takt!A6</f>
         <v>25000</v>
       </c>
-      <c r="B6" s="15">
+      <c r="B6" s="14">
         <f>Takt!B6</f>
         <v>9.6</v>
       </c>
-      <c r="C6" s="16">
-        <f>ROUNDUP(Inputs!$B$12/(B6*Inputs!$B$13),0)</f>
+      <c r="C6" s="15">
+        <f>ROUNDUP(Inputs!$B$10/(B6*Inputs!$B$11),0)</f>
         <v>111</v>
       </c>
-      <c r="D6" s="17">
+      <c r="D6" s="16">
         <f>Takt!E6</f>
         <v>7.68</v>
       </c>
-      <c r="E6" s="16">
-        <f>ROUNDUP(Inputs!$B$14/D6,0)</f>
+      <c r="E6" s="15">
+        <f>ROUNDUP(Inputs!$B$12/D6,0)</f>
         <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="16">
+      <c r="A7" s="15">
         <f>Takt!A7</f>
         <v>50000</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="14">
         <f>Takt!B7</f>
         <v>4.8</v>
       </c>
-      <c r="C7" s="16">
-        <f>ROUNDUP(Inputs!$B$12/(B7*Inputs!$B$13),0)</f>
+      <c r="C7" s="15">
+        <f>ROUNDUP(Inputs!$B$10/(B7*Inputs!$B$11),0)</f>
         <v>221</v>
       </c>
-      <c r="D7" s="17">
+      <c r="D7" s="16">
         <f>Takt!E7</f>
         <v>3.84</v>
       </c>
-      <c r="E7" s="16">
-        <f>ROUNDUP(Inputs!$B$14/D7,0)</f>
+      <c r="E7" s="15">
+        <f>ROUNDUP(Inputs!$B$12/D7,0)</f>
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="16">
+      <c r="A8" s="15">
         <f>Takt!A8</f>
         <v>100000</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="14">
         <f>Takt!B8</f>
         <v>2.4</v>
       </c>
-      <c r="C8" s="16">
-        <f>ROUNDUP(Inputs!$B$12/(B8*Inputs!$B$13),0)</f>
+      <c r="C8" s="15">
+        <f>ROUNDUP(Inputs!$B$10/(B8*Inputs!$B$11),0)</f>
         <v>442</v>
       </c>
-      <c r="D8" s="17">
+      <c r="D8" s="16">
         <f>Takt!E8</f>
         <v>1.92</v>
       </c>
-      <c r="E8" s="16">
-        <f>ROUNDUP(Inputs!$B$14/D8,0)</f>
+      <c r="E8" s="15">
+        <f>ROUNDUP(Inputs!$B$12/D8,0)</f>
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="20" t="s">
-        <v>73</v>
+      <c r="A10" s="19" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -1494,168 +1639,167 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B5" s="12">
+        <v>71</v>
+      </c>
+      <c r="B5" s="10">
         <v>1800</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="17">
         <v>1</v>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="20">
         <f>INT(B5/C5)</f>
         <v>1800</v>
       </c>
-      <c r="E5" s="22" t="str">
-        <f>IF(D5=$B$11,"◄ CONSTRAINT","")</f>
+      <c r="E5" s="21" t="str">
+        <f>IF(D5=$B$11,"Constraint","")</f>
         <v/>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="B6" s="12">
+        <v>72</v>
+      </c>
+      <c r="B6" s="10">
         <v>1300</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="17">
         <v>1</v>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="20">
         <f>INT(B6/C6)</f>
         <v>1300</v>
       </c>
-      <c r="E6" s="22" t="str">
-        <f>IF(D6=$B$11,"◄ CONSTRAINT","")</f>
+      <c r="E6" s="21" t="str">
+        <f>IF(D6=$B$11,"Constraint","")</f>
         <v/>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="B7" s="12">
+        <v>73</v>
+      </c>
+      <c r="B7" s="10">
         <v>1900</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="17">
         <v>2</v>
       </c>
-      <c r="D7" s="21">
+      <c r="D7" s="20">
         <f>INT(B7/C7)</f>
         <v>950</v>
       </c>
-      <c r="E7" s="22" t="str">
-        <f>IF(D7=$B$11,"◄ CONSTRAINT","")</f>
-        <v>◄ CONSTRAINT</v>
+      <c r="E7" s="21" t="str">
+        <f>IF(D7=$B$11,"Constraint","")</f>
+        <v>Constraint</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="B8" s="12">
+        <v>74</v>
+      </c>
+      <c r="B8" s="10">
         <v>2400</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="17">
         <v>2</v>
       </c>
-      <c r="D8" s="21">
+      <c r="D8" s="20">
         <f>INT(B8/C8)</f>
         <v>1200</v>
       </c>
-      <c r="E8" s="22" t="str">
-        <f>IF(D8=$B$11,"◄ CONSTRAINT","")</f>
+      <c r="E8" s="21" t="str">
+        <f>IF(D8=$B$11,"Constraint","")</f>
         <v/>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="B9" s="12">
+        <v>75</v>
+      </c>
+      <c r="B9" s="10">
         <v>1500</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="17">
         <v>1</v>
       </c>
-      <c r="D9" s="21">
+      <c r="D9" s="20">
         <f>INT(B9/C9)</f>
         <v>1500</v>
       </c>
-      <c r="E9" s="22" t="str">
-        <f>IF(D9=$B$11,"◄ CONSTRAINT","")</f>
+      <c r="E9" s="21" t="str">
+        <f>IF(D9=$B$11,"Constraint","")</f>
         <v/>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="B11" s="13">
+        <v>76</v>
+      </c>
+      <c r="B11" s="11">
         <f>MIN(D5:D9)</f>
         <v>950</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="B12" s="16">
+        <v>77</v>
+      </c>
+      <c r="B12" s="15">
         <f>Takt!A5/Inputs!B5*5</f>
         <v>200</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="B13" s="19">
+        <v>78</v>
+      </c>
+      <c r="B13" s="18">
         <f>B11/B12</f>
         <v>4.75</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="20" t="s">
-        <v>89</v>
+      <c r="A15" s="19" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
     <col min="2" max="3" width="15" customWidth="1"/>
@@ -1666,41 +1810,41 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="B4" s="12">
+        <v>82</v>
+      </c>
+      <c r="B4" s="10">
         <v>1200</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="B5" s="10">
+        <v>83</v>
+      </c>
+      <c r="B5" s="17">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="B6" s="12">
+        <v>84</v>
+      </c>
+      <c r="B6" s="10">
         <v>200</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B7" s="7">
         <v>6</v>
@@ -1708,354 +1852,353 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="B8" s="23">
+        <v>86</v>
+      </c>
+      <c r="B8" s="22">
         <v>450</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="10">
+      <c r="A11" s="17">
         <v>1</v>
       </c>
-      <c r="B11" s="21">
+      <c r="B11" s="20">
         <f t="shared" ref="B11:B22" si="0">$B$6</f>
         <v>200</v>
       </c>
-      <c r="C11" s="21">
+      <c r="C11" s="20">
         <f t="shared" ref="C11:C22" si="1">IF(A11&lt;$B$7,B11*$B$5,0)</f>
         <v>400</v>
       </c>
-      <c r="D11" s="12">
-        <v>0</v>
-      </c>
-      <c r="E11" s="21">
+      <c r="D11" s="10">
+        <v>0</v>
+      </c>
+      <c r="E11" s="20">
         <f>MAX(0,$B$4+D11-C11)</f>
         <v>800</v>
       </c>
-      <c r="F11" s="21">
+      <c r="F11" s="20">
         <f>MAX(0,C11-($B$4+D11))</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="10">
+      <c r="A12" s="17">
         <v>2</v>
       </c>
-      <c r="B12" s="21">
+      <c r="B12" s="20">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
-      <c r="C12" s="21">
+      <c r="C12" s="20">
         <f t="shared" si="1"/>
         <v>400</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="10">
         <v>400</v>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="20">
         <f t="shared" ref="E12:E22" si="2">MAX(0,E11+D12-C12)</f>
         <v>800</v>
       </c>
-      <c r="F12" s="21">
+      <c r="F12" s="20">
         <f t="shared" ref="F12:F22" si="3">MAX(0,C12-(E11+D12))</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="10">
+      <c r="A13" s="17">
         <v>3</v>
       </c>
-      <c r="B13" s="21">
+      <c r="B13" s="20">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
-      <c r="C13" s="21">
+      <c r="C13" s="20">
         <f t="shared" si="1"/>
         <v>400</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="10">
         <v>400</v>
       </c>
-      <c r="E13" s="21">
+      <c r="E13" s="20">
         <f t="shared" si="2"/>
         <v>800</v>
       </c>
-      <c r="F13" s="21">
+      <c r="F13" s="20">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="10">
+      <c r="A14" s="17">
         <v>4</v>
       </c>
-      <c r="B14" s="21">
+      <c r="B14" s="20">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
-      <c r="C14" s="21">
+      <c r="C14" s="20">
         <f t="shared" si="1"/>
         <v>400</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="10">
         <v>400</v>
       </c>
-      <c r="E14" s="21">
+      <c r="E14" s="20">
         <f t="shared" si="2"/>
         <v>800</v>
       </c>
-      <c r="F14" s="21">
+      <c r="F14" s="20">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" s="10">
+      <c r="A15" s="17">
         <v>5</v>
       </c>
-      <c r="B15" s="21">
+      <c r="B15" s="20">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
-      <c r="C15" s="21">
+      <c r="C15" s="20">
         <f t="shared" si="1"/>
         <v>400</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="10">
         <v>400</v>
       </c>
-      <c r="E15" s="21">
+      <c r="E15" s="20">
         <f t="shared" si="2"/>
         <v>800</v>
       </c>
-      <c r="F15" s="21">
+      <c r="F15" s="20">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="10">
+      <c r="A16" s="17">
         <v>6</v>
       </c>
-      <c r="B16" s="21">
+      <c r="B16" s="20">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
-      <c r="C16" s="21">
+      <c r="C16" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="10">
         <v>400</v>
       </c>
-      <c r="E16" s="21">
+      <c r="E16" s="20">
         <f t="shared" si="2"/>
         <v>1200</v>
       </c>
-      <c r="F16" s="21">
+      <c r="F16" s="20">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="10">
+      <c r="A17" s="17">
         <v>7</v>
       </c>
-      <c r="B17" s="21">
+      <c r="B17" s="20">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
-      <c r="C17" s="21">
+      <c r="C17" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D17" s="12">
-        <v>0</v>
-      </c>
-      <c r="E17" s="21">
+      <c r="D17" s="10">
+        <v>0</v>
+      </c>
+      <c r="E17" s="20">
         <f t="shared" si="2"/>
         <v>1200</v>
       </c>
-      <c r="F17" s="21">
+      <c r="F17" s="20">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="10">
+      <c r="A18" s="17">
         <v>8</v>
       </c>
-      <c r="B18" s="21">
+      <c r="B18" s="20">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
-      <c r="C18" s="21">
+      <c r="C18" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D18" s="12">
-        <v>0</v>
-      </c>
-      <c r="E18" s="21">
+      <c r="D18" s="10">
+        <v>0</v>
+      </c>
+      <c r="E18" s="20">
         <f t="shared" si="2"/>
         <v>1200</v>
       </c>
-      <c r="F18" s="21">
+      <c r="F18" s="20">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" s="10">
+      <c r="A19" s="17">
         <v>9</v>
       </c>
-      <c r="B19" s="21">
+      <c r="B19" s="20">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
-      <c r="C19" s="21">
+      <c r="C19" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D19" s="12">
-        <v>0</v>
-      </c>
-      <c r="E19" s="21">
+      <c r="D19" s="10">
+        <v>0</v>
+      </c>
+      <c r="E19" s="20">
         <f t="shared" si="2"/>
         <v>1200</v>
       </c>
-      <c r="F19" s="21">
+      <c r="F19" s="20">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" s="10">
+      <c r="A20" s="17">
         <v>10</v>
       </c>
-      <c r="B20" s="21">
+      <c r="B20" s="20">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
-      <c r="C20" s="21">
+      <c r="C20" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D20" s="12">
-        <v>0</v>
-      </c>
-      <c r="E20" s="21">
+      <c r="D20" s="10">
+        <v>0</v>
+      </c>
+      <c r="E20" s="20">
         <f t="shared" si="2"/>
         <v>1200</v>
       </c>
-      <c r="F20" s="21">
+      <c r="F20" s="20">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="10">
+      <c r="A21" s="17">
         <v>11</v>
       </c>
-      <c r="B21" s="21">
+      <c r="B21" s="20">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
-      <c r="C21" s="21">
+      <c r="C21" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D21" s="12">
-        <v>0</v>
-      </c>
-      <c r="E21" s="21">
+      <c r="D21" s="10">
+        <v>0</v>
+      </c>
+      <c r="E21" s="20">
         <f t="shared" si="2"/>
         <v>1200</v>
       </c>
-      <c r="F21" s="21">
+      <c r="F21" s="20">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" s="10">
+      <c r="A22" s="17">
         <v>12</v>
       </c>
-      <c r="B22" s="21">
+      <c r="B22" s="20">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
-      <c r="C22" s="21">
+      <c r="C22" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D22" s="12">
-        <v>0</v>
-      </c>
-      <c r="E22" s="21">
+      <c r="D22" s="10">
+        <v>0</v>
+      </c>
+      <c r="E22" s="20">
         <f t="shared" si="2"/>
         <v>1200</v>
       </c>
-      <c r="F22" s="21">
+      <c r="F22" s="20">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B24" s="21">
+        <v>93</v>
+      </c>
+      <c r="B24" s="20">
         <f>SUM(F11:F22)</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="B25" s="13">
+        <v>94</v>
+      </c>
+      <c r="B25" s="11">
         <f>INDEX(E11:E22,12)</f>
         <v>1200</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B26" s="24">
+        <v>95</v>
+      </c>
+      <c r="B26" s="23">
         <f>B25*B8</f>
         <v>540000</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28" s="20" t="s">
-        <v>106</v>
+      <c r="A28" s="19" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>